<commit_message>
Cargar datos crudos OSIPTEL en PostgreSQL
</commit_message>
<xml_diff>
--- a/datos/raw/4. COBERTURA VOZ MÓVIL.xlsx
+++ b/datos/raw/4. COBERTURA VOZ MÓVIL.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\2019\FINANZAS\PROCESAMIENTO DE INFORMACIÓN\21. DATOS ABIERTOS\2019-III\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian M\Documents\analisis-cobertura-movil-peru\datos\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_6B748AA2D1558F928BCF1BCE058E5EDD972646BA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11235"/>
+    <workbookView xWindow="12810" yWindow="2895" windowWidth="20280" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -105,9 +106,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="24" x14ac:knownFonts="1">
     <font>
@@ -653,18 +654,18 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -684,7 +685,7 @@
     <xf numFmtId="0" fontId="21" fillId="34" borderId="10" xfId="41" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="22" fillId="0" borderId="0" xfId="46" applyFont="1"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="46" applyFont="1"/>
   </cellXfs>
   <cellStyles count="47">
     <cellStyle name="20% - Énfasis1" xfId="18" builtinId="30" customBuiltin="1"/>
@@ -705,7 +706,7 @@
     <cellStyle name="60% - Énfasis4" xfId="32" builtinId="44" customBuiltin="1"/>
     <cellStyle name="60% - Énfasis5" xfId="36" builtinId="48" customBuiltin="1"/>
     <cellStyle name="60% - Énfasis6" xfId="40" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Buena" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
     <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
@@ -722,11 +723,11 @@
     <cellStyle name="Millares" xfId="46" builtinId="3"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="42"/>
-    <cellStyle name="Normal 3" xfId="44"/>
-    <cellStyle name="Normal 4" xfId="41"/>
-    <cellStyle name="Notas 2" xfId="43"/>
-    <cellStyle name="Porcentaje 2" xfId="45"/>
+    <cellStyle name="Normal 2" xfId="42" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="Normal 3" xfId="44" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="Normal 4" xfId="41" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Notas 2" xfId="43" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="Porcentaje 2" xfId="45" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
     <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto explicativo" xfId="15" builtinId="53" customBuiltin="1"/>
@@ -1010,7 +1011,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:I101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2406,13 +2407,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:E101"/>
+  <autoFilter ref="B4:E101" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B4:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>